<commit_message>
📊 BIST Screener | 03.04.2026 16:30 | 604 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-03.xlsx
+++ b/data/bist_screener_2026-04-03.xlsx
@@ -25615,42 +25615,40 @@
     <row r="579">
       <c r="A579" s="5" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B579" s="6" t="n">
-        <v>17.05</v>
+        <v>2.94</v>
       </c>
       <c r="C579" s="7" t="n">
-        <v>-0.0145</v>
+        <v>-0.05769999999999999</v>
       </c>
       <c r="D579" s="8" t="n">
-        <v>12240000</v>
+        <v>23190000</v>
       </c>
       <c r="E579" s="7" t="n">
-        <v>0.9246</v>
+        <v>0.1672</v>
       </c>
       <c r="F579" s="6" t="n">
-        <v>43.93</v>
-      </c>
-      <c r="G579" s="6" t="n">
-        <v>161.15</v>
-      </c>
+        <v>51.62</v>
+      </c>
+      <c r="G579" s="5" t="inlineStr"/>
       <c r="H579" s="5" t="inlineStr"/>
       <c r="I579" s="7" t="n">
-        <v>0.0028</v>
+        <v>-5.3262</v>
       </c>
       <c r="J579" s="7" t="n">
-        <v>-10.3171</v>
+        <v>-4.2562</v>
       </c>
       <c r="K579" s="5" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L579" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M579" s="5" t="inlineStr"/>
@@ -25658,21 +25656,21 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>13.23</v>
+        <v>5.8</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>0.0998</v>
+        <v>0.0105</v>
       </c>
       <c r="D580" s="9" t="n">
-        <v>122000000</v>
+        <v>10840000</v>
       </c>
       <c r="E580" s="2" t="inlineStr"/>
       <c r="F580" s="3" t="n">
-        <v>85.09999999999999</v>
+        <v>59.62</v>
       </c>
       <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
@@ -25683,44 +25681,44 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L580" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+      <c r="L580" s="2" t="inlineStr"/>
       <c r="M580" s="2" t="inlineStr"/>
     </row>
     <row r="581">
       <c r="A581" s="5" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B581" s="6" t="n">
-        <v>188.5</v>
+        <v>62.25</v>
       </c>
       <c r="C581" s="7" t="n">
-        <v>0.0357</v>
+        <v>0.0366</v>
       </c>
       <c r="D581" s="8" t="n">
-        <v>4820000</v>
-      </c>
-      <c r="E581" s="5" t="inlineStr"/>
+        <v>914380</v>
+      </c>
+      <c r="E581" s="7" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F581" s="6" t="n">
-        <v>63.58</v>
+        <v>60.57</v>
       </c>
       <c r="G581" s="5" t="inlineStr"/>
       <c r="H581" s="5" t="inlineStr"/>
       <c r="I581" s="5" t="inlineStr"/>
-      <c r="J581" s="5" t="inlineStr"/>
+      <c r="J581" s="7" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K581" s="5" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L581" s="5" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M581" s="5" t="inlineStr"/>
@@ -25728,36 +25726,38 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>3.56</v>
+        <v>2.68</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0.0379</v>
+        <v>0</v>
       </c>
       <c r="D582" s="9" t="n">
-        <v>51270000</v>
+        <v>98450000</v>
       </c>
       <c r="E582" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.6898000000000001</v>
       </c>
       <c r="F582" s="3" t="n">
-        <v>67.26000000000001</v>
+        <v>41.64</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
       <c r="I582" s="2" t="inlineStr"/>
-      <c r="J582" s="2" t="inlineStr"/>
+      <c r="J582" s="4" t="n">
+        <v>-2.0083</v>
+      </c>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L582" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M582" s="2" t="inlineStr"/>
@@ -25765,93 +25765,95 @@
     <row r="583">
       <c r="A583" s="5" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B583" s="6" t="n">
-        <v>17.4</v>
+        <v>88</v>
       </c>
       <c r="C583" s="7" t="n">
-        <v>0.0999</v>
+        <v>-0.0383</v>
       </c>
       <c r="D583" s="8" t="n">
-        <v>104120000</v>
-      </c>
-      <c r="E583" s="5" t="inlineStr"/>
+        <v>25790</v>
+      </c>
+      <c r="E583" s="7" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F583" s="6" t="n">
-        <v>58.99</v>
+        <v>42.39</v>
       </c>
       <c r="G583" s="5" t="inlineStr"/>
       <c r="H583" s="5" t="inlineStr"/>
-      <c r="I583" s="5" t="inlineStr"/>
-      <c r="J583" s="5" t="inlineStr"/>
+      <c r="I583" s="7" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J583" s="7" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K583" s="5" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L583" s="5" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L583" s="5" t="inlineStr"/>
       <c r="M583" s="5" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>8.449999999999999</v>
+        <v>35.76</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.009399999999999999</v>
+        <v>-0.0017</v>
       </c>
       <c r="D584" s="9" t="n">
-        <v>204180</v>
-      </c>
-      <c r="E584" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>5120000</v>
+      </c>
+      <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>45.09</v>
+        <v>46.1</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
-      <c r="I584" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J584" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I584" s="2" t="inlineStr"/>
+      <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L584" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L584" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="5" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B585" s="6" t="n">
-        <v>43.62</v>
+        <v>26.86</v>
       </c>
       <c r="C585" s="7" t="n">
-        <v>-0.0215</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="D585" s="8" t="n">
-        <v>30220000</v>
-      </c>
-      <c r="E585" s="5" t="inlineStr"/>
+        <v>17180000</v>
+      </c>
+      <c r="E585" s="7" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F585" s="6" t="n">
-        <v>60.67</v>
+        <v>50.98</v>
       </c>
       <c r="G585" s="5" t="inlineStr"/>
       <c r="H585" s="5" t="inlineStr"/>
@@ -25859,12 +25861,12 @@
       <c r="J585" s="5" t="inlineStr"/>
       <c r="K585" s="5" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L585" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M585" s="5" t="inlineStr"/>
@@ -25872,21 +25874,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ZGYO</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>58.25</v>
+        <v>26.84</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0372</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="D586" s="9" t="n">
-        <v>3320000</v>
+        <v>21270000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>43.98</v>
+        <v>54.14</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25894,12 +25896,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25907,21 +25909,21 @@
     <row r="587">
       <c r="A587" s="5" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B587" s="6" t="n">
-        <v>5.8</v>
+        <v>58.25</v>
       </c>
       <c r="C587" s="7" t="n">
-        <v>0.0105</v>
+        <v>-0.0372</v>
       </c>
       <c r="D587" s="8" t="n">
-        <v>10840000</v>
+        <v>3320000</v>
       </c>
       <c r="E587" s="5" t="inlineStr"/>
       <c r="F587" s="6" t="n">
-        <v>59.62</v>
+        <v>43.98</v>
       </c>
       <c r="G587" s="5" t="inlineStr"/>
       <c r="H587" s="5" t="inlineStr"/>
@@ -25929,43 +25931,53 @@
       <c r="J587" s="5" t="inlineStr"/>
       <c r="K587" s="5" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L587" s="5" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L587" s="5" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M587" s="5" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>2.81</v>
+        <v>121</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0977</v>
+        <v>-0.0171</v>
       </c>
       <c r="D588" s="9" t="n">
-        <v>202390000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>392200</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>45.23</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25973,21 +25985,23 @@
     <row r="589">
       <c r="A589" s="5" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B589" s="6" t="n">
-        <v>35.76</v>
+        <v>7.04</v>
       </c>
       <c r="C589" s="7" t="n">
-        <v>-0.0017</v>
+        <v>-0.0222</v>
       </c>
       <c r="D589" s="8" t="n">
-        <v>5120000</v>
-      </c>
-      <c r="E589" s="5" t="inlineStr"/>
+        <v>10330000</v>
+      </c>
+      <c r="E589" s="7" t="n">
+        <v>0.28</v>
+      </c>
       <c r="F589" s="6" t="n">
-        <v>46.1</v>
+        <v>35.11</v>
       </c>
       <c r="G589" s="5" t="inlineStr"/>
       <c r="H589" s="5" t="inlineStr"/>
@@ -25995,12 +26009,12 @@
       <c r="J589" s="5" t="inlineStr"/>
       <c r="K589" s="5" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M589" s="5" t="inlineStr"/>
@@ -26008,21 +26022,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>149.3</v>
+        <v>2.81</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.002</v>
-      </c>
-      <c r="D590" s="3" t="n">
-        <v>16220000</v>
+        <v>0.0977</v>
+      </c>
+      <c r="D590" s="9" t="n">
+        <v>202390000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>73.95999999999999</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26030,12 +26044,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26043,71 +26057,73 @@
     <row r="591">
       <c r="A591" s="5" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B591" s="6" t="n">
-        <v>88</v>
+        <v>43.62</v>
       </c>
       <c r="C591" s="7" t="n">
-        <v>-0.0383</v>
+        <v>-0.0215</v>
       </c>
       <c r="D591" s="8" t="n">
-        <v>25790</v>
-      </c>
-      <c r="E591" s="7" t="n">
-        <v>0.58</v>
-      </c>
+        <v>30220000</v>
+      </c>
+      <c r="E591" s="5" t="inlineStr"/>
       <c r="F591" s="6" t="n">
-        <v>42.39</v>
+        <v>60.67</v>
       </c>
       <c r="G591" s="5" t="inlineStr"/>
       <c r="H591" s="5" t="inlineStr"/>
-      <c r="I591" s="7" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J591" s="7" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I591" s="5" t="inlineStr"/>
+      <c r="J591" s="5" t="inlineStr"/>
       <c r="K591" s="5" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L591" s="5" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L591" s="5" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M591" s="5" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ZGYO</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>26.84</v>
+        <v>7.34</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.09939999999999999</v>
       </c>
       <c r="D592" s="9" t="n">
-        <v>21270000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>101610000</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.2478</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>54.14</v>
+        <v>15.9</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26115,79 +26131,79 @@
     <row r="593">
       <c r="A593" s="5" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B593" s="6" t="n">
-        <v>7.34</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="C593" s="7" t="n">
-        <v>-0.09939999999999999</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="D593" s="8" t="n">
-        <v>101610000</v>
+        <v>204180</v>
       </c>
       <c r="E593" s="7" t="n">
-        <v>0.2478</v>
+        <v>0.95</v>
       </c>
       <c r="F593" s="6" t="n">
-        <v>15.9</v>
+        <v>45.09</v>
       </c>
       <c r="G593" s="5" t="inlineStr"/>
       <c r="H593" s="5" t="inlineStr"/>
       <c r="I593" s="7" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J593" s="5" t="inlineStr"/>
+        <v>-23.6291</v>
+      </c>
+      <c r="J593" s="7" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K593" s="5" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L593" s="5" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="5" t="inlineStr"/>
       <c r="M593" s="5" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>3.25</v>
+        <v>17.05</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.098</v>
+        <v>-0.0145</v>
       </c>
       <c r="D594" s="9" t="n">
-        <v>40940000</v>
+        <v>12240000</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.9246</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>68.34999999999999</v>
-      </c>
-      <c r="G594" s="2" t="inlineStr"/>
+        <v>43.93</v>
+      </c>
+      <c r="G594" s="3" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="4" t="n">
-        <v>-191.6342</v>
+        <v>0.0028</v>
       </c>
       <c r="J594" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-10.3171</v>
       </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26195,34 +26211,40 @@
     <row r="595">
       <c r="A595" s="5" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B595" s="6" t="n">
-        <v>14.69</v>
+        <v>3.25</v>
       </c>
       <c r="C595" s="7" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.098</v>
       </c>
       <c r="D595" s="8" t="n">
-        <v>76800000</v>
-      </c>
-      <c r="E595" s="5" t="inlineStr"/>
+        <v>40940000</v>
+      </c>
+      <c r="E595" s="7" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F595" s="6" t="n">
-        <v>60.1</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="G595" s="5" t="inlineStr"/>
       <c r="H595" s="5" t="inlineStr"/>
-      <c r="I595" s="5" t="inlineStr"/>
-      <c r="J595" s="5" t="inlineStr"/>
+      <c r="I595" s="7" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J595" s="7" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K595" s="5" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L595" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="5" t="inlineStr"/>
@@ -26230,40 +26252,34 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>121</v>
+        <v>17.4</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0171</v>
+        <v>0.0999</v>
       </c>
       <c r="D596" s="9" t="n">
-        <v>392200</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>104120000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>45.23</v>
+        <v>58.99</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26271,21 +26287,21 @@
     <row r="597">
       <c r="A597" s="5" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B597" s="6" t="n">
-        <v>24</v>
+        <v>32.2</v>
       </c>
       <c r="C597" s="7" t="n">
-        <v>0.0127</v>
+        <v>0.0019</v>
       </c>
       <c r="D597" s="8" t="n">
-        <v>20280000</v>
+        <v>5320000</v>
       </c>
       <c r="E597" s="5" t="inlineStr"/>
       <c r="F597" s="6" t="n">
-        <v>55.99</v>
+        <v>50.65</v>
       </c>
       <c r="G597" s="5" t="inlineStr"/>
       <c r="H597" s="5" t="inlineStr"/>
@@ -26293,12 +26309,12 @@
       <c r="J597" s="5" t="inlineStr"/>
       <c r="K597" s="5" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L597" s="5" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M597" s="5" t="inlineStr"/>
@@ -26306,21 +26322,21 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>32.2</v>
+        <v>14.69</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D598" s="9" t="n">
-        <v>5320000</v>
+        <v>76800000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>50.65</v>
+        <v>60.1</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26328,12 +26344,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26341,40 +26357,34 @@
     <row r="599">
       <c r="A599" s="5" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B599" s="6" t="n">
-        <v>2.94</v>
+        <v>24</v>
       </c>
       <c r="C599" s="7" t="n">
-        <v>-0.05769999999999999</v>
+        <v>0.0127</v>
       </c>
       <c r="D599" s="8" t="n">
-        <v>23190000</v>
-      </c>
-      <c r="E599" s="7" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>20280000</v>
+      </c>
+      <c r="E599" s="5" t="inlineStr"/>
       <c r="F599" s="6" t="n">
-        <v>51.62</v>
+        <v>55.99</v>
       </c>
       <c r="G599" s="5" t="inlineStr"/>
       <c r="H599" s="5" t="inlineStr"/>
-      <c r="I599" s="7" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J599" s="7" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I599" s="5" t="inlineStr"/>
+      <c r="J599" s="5" t="inlineStr"/>
       <c r="K599" s="5" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L599" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M599" s="5" t="inlineStr"/>
@@ -26382,23 +26392,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>241</v>
+        <v>13.23</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0123</v>
+        <v>0.0998</v>
       </c>
       <c r="D600" s="9" t="n">
-        <v>9230</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>122000000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>36.37</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26406,32 +26414,34 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="5" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B601" s="6" t="n">
-        <v>26.86</v>
+        <v>188.5</v>
       </c>
       <c r="C601" s="7" t="n">
-        <v>-0.009599999999999999</v>
+        <v>0.0357</v>
       </c>
       <c r="D601" s="8" t="n">
-        <v>17180000</v>
-      </c>
-      <c r="E601" s="7" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>4820000</v>
+      </c>
+      <c r="E601" s="5" t="inlineStr"/>
       <c r="F601" s="6" t="n">
-        <v>50.98</v>
+        <v>63.58</v>
       </c>
       <c r="G601" s="5" t="inlineStr"/>
       <c r="H601" s="5" t="inlineStr"/>
@@ -26444,7 +26454,7 @@
       </c>
       <c r="L601" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M601" s="5" t="inlineStr"/>
@@ -26452,89 +26462,81 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>2.68</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0</v>
+        <v>-0.0043</v>
       </c>
       <c r="D602" s="9" t="n">
-        <v>98450000</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.6898000000000001</v>
-      </c>
+        <v>18310000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>41.64</v>
+        <v>42.91</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="4" t="n">
-        <v>-2.0083</v>
-      </c>
-      <c r="K602" s="2" t="inlineStr">
-        <is>
-          <t>Tüketici hizmetleri</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="J602" s="2" t="inlineStr"/>
+      <c r="K602" s="2" t="inlineStr"/>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="5" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B603" s="6" t="n">
-        <v>82.40000000000001</v>
+        <v>241</v>
       </c>
       <c r="C603" s="7" t="n">
-        <v>-0.0043</v>
+        <v>-0.0123</v>
       </c>
       <c r="D603" s="8" t="n">
-        <v>18310000</v>
-      </c>
-      <c r="E603" s="5" t="inlineStr"/>
+        <v>9230</v>
+      </c>
+      <c r="E603" s="7" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F603" s="6" t="n">
-        <v>42.91</v>
+        <v>36.37</v>
       </c>
       <c r="G603" s="5" t="inlineStr"/>
       <c r="H603" s="5" t="inlineStr"/>
       <c r="I603" s="5" t="inlineStr"/>
       <c r="J603" s="5" t="inlineStr"/>
-      <c r="K603" s="5" t="inlineStr"/>
+      <c r="K603" s="5" t="inlineStr">
+        <is>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
       <c r="L603" s="5" t="inlineStr"/>
       <c r="M603" s="5" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>7.04</v>
+        <v>149.3</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0222</v>
-      </c>
-      <c r="D604" s="9" t="n">
-        <v>10330000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.28</v>
-      </c>
+        <v>-0.002</v>
+      </c>
+      <c r="D604" s="3" t="n">
+        <v>16220000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>35.11</v>
+        <v>73.95999999999999</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26542,12 +26544,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26555,38 +26557,36 @@
     <row r="605">
       <c r="A605" s="5" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B605" s="6" t="n">
-        <v>62.25</v>
+        <v>3.56</v>
       </c>
       <c r="C605" s="7" t="n">
-        <v>0.0366</v>
+        <v>0.0379</v>
       </c>
       <c r="D605" s="8" t="n">
-        <v>914380</v>
+        <v>51270000</v>
       </c>
       <c r="E605" s="7" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.8667</v>
       </c>
       <c r="F605" s="6" t="n">
-        <v>60.57</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="G605" s="5" t="inlineStr"/>
       <c r="H605" s="5" t="inlineStr"/>
       <c r="I605" s="5" t="inlineStr"/>
-      <c r="J605" s="7" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J605" s="5" t="inlineStr"/>
       <c r="K605" s="5" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L605" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="5" t="inlineStr"/>
@@ -26613,7 +26613,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>03.04.2026 15:30</t>
+          <t>03.04.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 03.04.2026 17:07 | 604 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-03.xlsx
+++ b/data/bist_screener_2026-04-03.xlsx
@@ -25615,40 +25615,34 @@
     <row r="579">
       <c r="A579" s="5" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B579" s="6" t="n">
-        <v>2.94</v>
+        <v>24</v>
       </c>
       <c r="C579" s="7" t="n">
-        <v>-0.05769999999999999</v>
+        <v>0.0127</v>
       </c>
       <c r="D579" s="8" t="n">
-        <v>23190000</v>
-      </c>
-      <c r="E579" s="7" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>20280000</v>
+      </c>
+      <c r="E579" s="5" t="inlineStr"/>
       <c r="F579" s="6" t="n">
-        <v>51.62</v>
+        <v>55.99</v>
       </c>
       <c r="G579" s="5" t="inlineStr"/>
       <c r="H579" s="5" t="inlineStr"/>
-      <c r="I579" s="7" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J579" s="7" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I579" s="5" t="inlineStr"/>
+      <c r="J579" s="5" t="inlineStr"/>
       <c r="K579" s="5" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L579" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M579" s="5" t="inlineStr"/>
@@ -25656,21 +25650,21 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>5.8</v>
+        <v>17.4</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>0.0105</v>
+        <v>0.0999</v>
       </c>
       <c r="D580" s="9" t="n">
-        <v>10840000</v>
+        <v>104120000</v>
       </c>
       <c r="E580" s="2" t="inlineStr"/>
       <c r="F580" s="3" t="n">
-        <v>59.62</v>
+        <v>58.99</v>
       </c>
       <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
@@ -25681,44 +25675,44 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L580" s="2" t="inlineStr"/>
+      <c r="L580" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M580" s="2" t="inlineStr"/>
     </row>
     <row r="581">
       <c r="A581" s="5" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B581" s="6" t="n">
-        <v>62.25</v>
+        <v>149.3</v>
       </c>
       <c r="C581" s="7" t="n">
-        <v>0.0366</v>
-      </c>
-      <c r="D581" s="8" t="n">
-        <v>914380</v>
-      </c>
-      <c r="E581" s="7" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>-0.002</v>
+      </c>
+      <c r="D581" s="6" t="n">
+        <v>16220000</v>
+      </c>
+      <c r="E581" s="5" t="inlineStr"/>
       <c r="F581" s="6" t="n">
-        <v>60.57</v>
+        <v>73.95999999999999</v>
       </c>
       <c r="G581" s="5" t="inlineStr"/>
       <c r="H581" s="5" t="inlineStr"/>
       <c r="I581" s="5" t="inlineStr"/>
-      <c r="J581" s="7" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J581" s="5" t="inlineStr"/>
       <c r="K581" s="5" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L581" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M581" s="5" t="inlineStr"/>
@@ -25726,38 +25720,36 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>2.68</v>
+        <v>26.86</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="D582" s="9" t="n">
-        <v>98450000</v>
+        <v>17180000</v>
       </c>
       <c r="E582" s="4" t="n">
-        <v>0.6898000000000001</v>
+        <v>0.2667</v>
       </c>
       <c r="F582" s="3" t="n">
-        <v>41.64</v>
+        <v>50.98</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
       <c r="I582" s="2" t="inlineStr"/>
-      <c r="J582" s="4" t="n">
-        <v>-2.0083</v>
-      </c>
+      <c r="J582" s="2" t="inlineStr"/>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L582" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M582" s="2" t="inlineStr"/>
@@ -25765,35 +25757,31 @@
     <row r="583">
       <c r="A583" s="5" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B583" s="6" t="n">
-        <v>88</v>
+        <v>241</v>
       </c>
       <c r="C583" s="7" t="n">
-        <v>-0.0383</v>
+        <v>-0.0123</v>
       </c>
       <c r="D583" s="8" t="n">
-        <v>25790</v>
+        <v>9230</v>
       </c>
       <c r="E583" s="7" t="n">
-        <v>0.58</v>
+        <v>0.2578</v>
       </c>
       <c r="F583" s="6" t="n">
-        <v>42.39</v>
+        <v>36.37</v>
       </c>
       <c r="G583" s="5" t="inlineStr"/>
       <c r="H583" s="5" t="inlineStr"/>
-      <c r="I583" s="7" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J583" s="7" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I583" s="5" t="inlineStr"/>
+      <c r="J583" s="5" t="inlineStr"/>
       <c r="K583" s="5" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L583" s="5" t="inlineStr"/>
@@ -25802,34 +25790,38 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>35.76</v>
+        <v>2.68</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0017</v>
+        <v>0</v>
       </c>
       <c r="D584" s="9" t="n">
-        <v>5120000</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>98450000</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.6898000000000001</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>46.1</v>
+        <v>41.64</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="2" t="inlineStr"/>
+      <c r="J584" s="4" t="n">
+        <v>-2.0083</v>
+      </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25837,23 +25829,21 @@
     <row r="585">
       <c r="A585" s="5" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B585" s="6" t="n">
-        <v>26.86</v>
+        <v>35.76</v>
       </c>
       <c r="C585" s="7" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.0017</v>
       </c>
       <c r="D585" s="8" t="n">
-        <v>17180000</v>
-      </c>
-      <c r="E585" s="7" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>5120000</v>
+      </c>
+      <c r="E585" s="5" t="inlineStr"/>
       <c r="F585" s="6" t="n">
-        <v>50.98</v>
+        <v>46.1</v>
       </c>
       <c r="G585" s="5" t="inlineStr"/>
       <c r="H585" s="5" t="inlineStr"/>
@@ -25861,12 +25851,12 @@
       <c r="J585" s="5" t="inlineStr"/>
       <c r="K585" s="5" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L585" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M585" s="5" t="inlineStr"/>
@@ -25874,21 +25864,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>ZGYO</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>26.84</v>
+        <v>58.25</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.0372</v>
       </c>
       <c r="D586" s="9" t="n">
-        <v>21270000</v>
+        <v>3320000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>54.14</v>
+        <v>43.98</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25896,12 +25886,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25909,21 +25899,21 @@
     <row r="587">
       <c r="A587" s="5" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B587" s="6" t="n">
-        <v>58.25</v>
+        <v>14.69</v>
       </c>
       <c r="C587" s="7" t="n">
-        <v>-0.0372</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D587" s="8" t="n">
-        <v>3320000</v>
+        <v>76800000</v>
       </c>
       <c r="E587" s="5" t="inlineStr"/>
       <c r="F587" s="6" t="n">
-        <v>43.98</v>
+        <v>60.1</v>
       </c>
       <c r="G587" s="5" t="inlineStr"/>
       <c r="H587" s="5" t="inlineStr"/>
@@ -25931,12 +25921,12 @@
       <c r="J587" s="5" t="inlineStr"/>
       <c r="K587" s="5" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L587" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M587" s="5" t="inlineStr"/>
@@ -25944,40 +25934,36 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>121</v>
+        <v>3.56</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0171</v>
+        <v>0.0379</v>
       </c>
       <c r="D588" s="9" t="n">
-        <v>392200</v>
+        <v>51270000</v>
       </c>
       <c r="E588" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.8667</v>
       </c>
       <c r="F588" s="3" t="n">
-        <v>45.23</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25985,28 +25971,32 @@
     <row r="589">
       <c r="A589" s="5" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B589" s="6" t="n">
-        <v>7.04</v>
+        <v>2.94</v>
       </c>
       <c r="C589" s="7" t="n">
-        <v>-0.0222</v>
+        <v>-0.05769999999999999</v>
       </c>
       <c r="D589" s="8" t="n">
-        <v>10330000</v>
+        <v>23190000</v>
       </c>
       <c r="E589" s="7" t="n">
-        <v>0.28</v>
+        <v>0.1672</v>
       </c>
       <c r="F589" s="6" t="n">
-        <v>35.11</v>
+        <v>51.62</v>
       </c>
       <c r="G589" s="5" t="inlineStr"/>
       <c r="H589" s="5" t="inlineStr"/>
-      <c r="I589" s="5" t="inlineStr"/>
-      <c r="J589" s="5" t="inlineStr"/>
+      <c r="I589" s="7" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J589" s="7" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K589" s="5" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26014,7 +26004,7 @@
       </c>
       <c r="L589" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M589" s="5" t="inlineStr"/>
@@ -26022,21 +26012,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>2.81</v>
+        <v>188.5</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0977</v>
+        <v>0.0357</v>
       </c>
       <c r="D590" s="9" t="n">
-        <v>202390000</v>
+        <v>4820000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>63.58</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26044,12 +26034,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26057,21 +26047,21 @@
     <row r="591">
       <c r="A591" s="5" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B591" s="6" t="n">
-        <v>43.62</v>
+        <v>2.81</v>
       </c>
       <c r="C591" s="7" t="n">
-        <v>-0.0215</v>
+        <v>0.0977</v>
       </c>
       <c r="D591" s="8" t="n">
-        <v>30220000</v>
+        <v>202390000</v>
       </c>
       <c r="E591" s="5" t="inlineStr"/>
       <c r="F591" s="6" t="n">
-        <v>60.67</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G591" s="5" t="inlineStr"/>
       <c r="H591" s="5" t="inlineStr"/>
@@ -26079,12 +26069,12 @@
       <c r="J591" s="5" t="inlineStr"/>
       <c r="K591" s="5" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L591" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M591" s="5" t="inlineStr"/>
@@ -26092,118 +26082,104 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>7.34</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.09939999999999999</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="D592" s="9" t="n">
-        <v>101610000</v>
+        <v>204180</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.2478</v>
+        <v>0.95</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>15.9</v>
+        <v>45.09</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J592" s="2" t="inlineStr"/>
+        <v>-23.6291</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="5" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B593" s="6" t="n">
-        <v>8.449999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="C593" s="7" t="n">
-        <v>-0.009399999999999999</v>
+        <v>-0.0043</v>
       </c>
       <c r="D593" s="8" t="n">
-        <v>204180</v>
-      </c>
-      <c r="E593" s="7" t="n">
-        <v>0.95</v>
-      </c>
+        <v>18310000</v>
+      </c>
+      <c r="E593" s="5" t="inlineStr"/>
       <c r="F593" s="6" t="n">
-        <v>45.09</v>
+        <v>42.91</v>
       </c>
       <c r="G593" s="5" t="inlineStr"/>
       <c r="H593" s="5" t="inlineStr"/>
-      <c r="I593" s="7" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J593" s="7" t="n">
-        <v>-0.4678</v>
-      </c>
-      <c r="K593" s="5" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
+      <c r="I593" s="5" t="inlineStr"/>
+      <c r="J593" s="5" t="inlineStr"/>
+      <c r="K593" s="5" t="inlineStr"/>
       <c r="L593" s="5" t="inlineStr"/>
       <c r="M593" s="5" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>17.05</v>
+        <v>121</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0145</v>
+        <v>-0.0171</v>
       </c>
       <c r="D594" s="9" t="n">
-        <v>12240000</v>
+        <v>392200</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.1071</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>43.93</v>
-      </c>
-      <c r="G594" s="3" t="n">
-        <v>161.15</v>
-      </c>
+        <v>45.23</v>
+      </c>
+      <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="4" t="n">
-        <v>0.0028</v>
+        <v>-3.6635</v>
       </c>
       <c r="J594" s="4" t="n">
-        <v>-10.3171</v>
+        <v>-0.4897</v>
       </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26211,40 +26187,38 @@
     <row r="595">
       <c r="A595" s="5" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B595" s="6" t="n">
-        <v>3.25</v>
+        <v>62.25</v>
       </c>
       <c r="C595" s="7" t="n">
-        <v>0.098</v>
+        <v>0.0366</v>
       </c>
       <c r="D595" s="8" t="n">
-        <v>40940000</v>
+        <v>914380</v>
       </c>
       <c r="E595" s="7" t="n">
-        <v>0.7119</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F595" s="6" t="n">
-        <v>68.34999999999999</v>
+        <v>60.57</v>
       </c>
       <c r="G595" s="5" t="inlineStr"/>
       <c r="H595" s="5" t="inlineStr"/>
-      <c r="I595" s="7" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I595" s="5" t="inlineStr"/>
       <c r="J595" s="7" t="n">
-        <v>-0.8093</v>
+        <v>0.4139</v>
       </c>
       <c r="K595" s="5" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L595" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="5" t="inlineStr"/>
@@ -26252,34 +26226,40 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>17.4</v>
+        <v>3.25</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0999</v>
+        <v>0.098</v>
       </c>
       <c r="D596" s="9" t="n">
-        <v>104120000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>40940000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>58.99</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26287,21 +26267,21 @@
     <row r="597">
       <c r="A597" s="5" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B597" s="6" t="n">
-        <v>32.2</v>
+        <v>43.62</v>
       </c>
       <c r="C597" s="7" t="n">
-        <v>0.0019</v>
+        <v>-0.0215</v>
       </c>
       <c r="D597" s="8" t="n">
-        <v>5320000</v>
+        <v>30220000</v>
       </c>
       <c r="E597" s="5" t="inlineStr"/>
       <c r="F597" s="6" t="n">
-        <v>50.65</v>
+        <v>60.67</v>
       </c>
       <c r="G597" s="5" t="inlineStr"/>
       <c r="H597" s="5" t="inlineStr"/>
@@ -26309,12 +26289,12 @@
       <c r="J597" s="5" t="inlineStr"/>
       <c r="K597" s="5" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L597" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M597" s="5" t="inlineStr"/>
@@ -26322,21 +26302,21 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>14.69</v>
+        <v>5.8</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0105</v>
       </c>
       <c r="D598" s="9" t="n">
-        <v>76800000</v>
+        <v>10840000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>60.1</v>
+        <v>59.62</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26344,82 +26324,84 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="5" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B599" s="6" t="n">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="C599" s="7" t="n">
-        <v>0.0127</v>
+        <v>-0.0383</v>
       </c>
       <c r="D599" s="8" t="n">
-        <v>20280000</v>
-      </c>
-      <c r="E599" s="5" t="inlineStr"/>
+        <v>25790</v>
+      </c>
+      <c r="E599" s="7" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F599" s="6" t="n">
-        <v>55.99</v>
+        <v>42.39</v>
       </c>
       <c r="G599" s="5" t="inlineStr"/>
       <c r="H599" s="5" t="inlineStr"/>
-      <c r="I599" s="5" t="inlineStr"/>
-      <c r="J599" s="5" t="inlineStr"/>
+      <c r="I599" s="7" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J599" s="7" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K599" s="5" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L599" s="5" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L599" s="5" t="inlineStr"/>
       <c r="M599" s="5" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>13.23</v>
+        <v>7.34</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0998</v>
+        <v>-0.09939999999999999</v>
       </c>
       <c r="D600" s="9" t="n">
-        <v>122000000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>101610000</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.2478</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>85.09999999999999</v>
+        <v>15.9</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26427,21 +26409,21 @@
     <row r="601">
       <c r="A601" s="5" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ZGYO</t>
         </is>
       </c>
       <c r="B601" s="6" t="n">
-        <v>188.5</v>
+        <v>26.84</v>
       </c>
       <c r="C601" s="7" t="n">
-        <v>0.0357</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="D601" s="8" t="n">
-        <v>4820000</v>
+        <v>21270000</v>
       </c>
       <c r="E601" s="5" t="inlineStr"/>
       <c r="F601" s="6" t="n">
-        <v>63.58</v>
+        <v>54.14</v>
       </c>
       <c r="G601" s="5" t="inlineStr"/>
       <c r="H601" s="5" t="inlineStr"/>
@@ -26449,12 +26431,12 @@
       <c r="J601" s="5" t="inlineStr"/>
       <c r="K601" s="5" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L601" s="5" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="5" t="inlineStr"/>
@@ -26462,50 +26444,58 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>82.40000000000001</v>
+        <v>7.04</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0043</v>
+        <v>-0.0222</v>
       </c>
       <c r="D602" s="9" t="n">
-        <v>18310000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>10330000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.28</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>42.91</v>
+        <v>35.11</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr"/>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="5" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B603" s="6" t="n">
-        <v>241</v>
+        <v>13.23</v>
       </c>
       <c r="C603" s="7" t="n">
-        <v>-0.0123</v>
+        <v>0.0998</v>
       </c>
       <c r="D603" s="8" t="n">
-        <v>9230</v>
-      </c>
-      <c r="E603" s="7" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>122000000</v>
+      </c>
+      <c r="E603" s="5" t="inlineStr"/>
       <c r="F603" s="6" t="n">
-        <v>36.37</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="G603" s="5" t="inlineStr"/>
       <c r="H603" s="5" t="inlineStr"/>
@@ -26513,30 +26503,34 @@
       <c r="J603" s="5" t="inlineStr"/>
       <c r="K603" s="5" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="5" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="5" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="5" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>149.3</v>
+        <v>32.2</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.002</v>
-      </c>
-      <c r="D604" s="3" t="n">
-        <v>16220000</v>
+        <v>0.0019</v>
+      </c>
+      <c r="D604" s="9" t="n">
+        <v>5320000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>73.95999999999999</v>
+        <v>50.65</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26544,12 +26538,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26557,36 +26551,42 @@
     <row r="605">
       <c r="A605" s="5" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B605" s="6" t="n">
-        <v>3.56</v>
+        <v>17.05</v>
       </c>
       <c r="C605" s="7" t="n">
-        <v>0.0379</v>
+        <v>-0.0145</v>
       </c>
       <c r="D605" s="8" t="n">
-        <v>51270000</v>
+        <v>12240000</v>
       </c>
       <c r="E605" s="7" t="n">
-        <v>0.8667</v>
+        <v>0.9246</v>
       </c>
       <c r="F605" s="6" t="n">
-        <v>67.26000000000001</v>
-      </c>
-      <c r="G605" s="5" t="inlineStr"/>
+        <v>43.93</v>
+      </c>
+      <c r="G605" s="6" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H605" s="5" t="inlineStr"/>
-      <c r="I605" s="5" t="inlineStr"/>
-      <c r="J605" s="5" t="inlineStr"/>
+      <c r="I605" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J605" s="7" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K605" s="5" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L605" s="5" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M605" s="5" t="inlineStr"/>
@@ -26613,7 +26613,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>03.04.2026 16:30</t>
+          <t>03.04.2026 17:07</t>
         </is>
       </c>
     </row>

</xml_diff>